<commit_message>
Update beverage ORD names across Kobo and exports
</commit_message>
<xml_diff>
--- a/templates/template_by_dealer.xlsx
+++ b/templates/template_by_dealer.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simaple_form" sheetId="1" r:id="R84f0cca44ac74fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simaple_form" sheetId="1" r:id="R22278b7ba29a46f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,33 +79,12 @@
     <x:t xml:space="preserve">WURKZ</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">CAMBODIA ED</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DAZZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DAZZ Zero Sugar</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">IZE PET 300ml Flavour</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">IZE COLA PET 1.5L All SKUs</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">EXPREZ Melon</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Wurkz Ice</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CAMBODIA Sport 300mL</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CAMBODIA Sport 500mL</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CAMBODIA WATER 500mL</x:t>
   </x:si>
   <x:si>
@@ -169,27 +148,6 @@
     <x:t xml:space="preserve">Coca Cola 330ml</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Boostrong</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Krud ED</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Champion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">King Kong Ice</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Krud Ice</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Super Boostrong</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">King Kong</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">AIRA</x:t>
   </x:si>
   <x:si>
@@ -217,19 +175,10 @@
     <x:t xml:space="preserve">Big Cola 3L</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">EXPREZ Can 330ml</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Sting Can 330ml</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Idol Can 330ml</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CAMBODIA Sport 500ml</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CAMBODIA Sport 300ml</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pocari Sweat</x:t>
@@ -457,13 +406,13 @@
     <xdr:ext cx="809625" cy="809625"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc65273874dde46c9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra885a6d504c24f93"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1127,8 +1076,8 @@
       <x:c r="A14" s="3">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="s">
-        <x:v>23</x:v>
+      <x:c r="B14" s="1" t="str">
+        <x:v>CAMBODIA ED ORD</x:v>
       </x:c>
       <x:c r="C14" s="10"/>
       <x:c r="D14" s="11"/>
@@ -1160,8 +1109,8 @@
       <x:c r="A15" s="3">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B15" s="1" t="s">
-        <x:v>24</x:v>
+      <x:c r="B15" s="1" t="str">
+        <x:v>DAZZ ORD</x:v>
       </x:c>
       <x:c r="C15" s="10"/>
       <x:c r="D15" s="11"/>
@@ -1193,8 +1142,8 @@
       <x:c r="A16" s="3">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B16" s="1" t="s">
-        <x:v>25</x:v>
+      <x:c r="B16" s="1" t="str">
+        <x:v>DAZZ Zero Sugar ORD</x:v>
       </x:c>
       <x:c r="C16" s="10"/>
       <x:c r="D16" s="11"/>
@@ -1227,7 +1176,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C17" s="10"/>
       <x:c r="D17" s="11"/>
@@ -1260,7 +1209,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C18" s="10"/>
       <x:c r="D18" s="11"/>
@@ -1292,8 +1241,8 @@
       <x:c r="A19" s="3">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B19" s="1" t="s">
-        <x:v>28</x:v>
+      <x:c r="B19" s="1" t="str">
+        <x:v>EXPREZ Melon ORD</x:v>
       </x:c>
       <x:c r="C19" s="10"/>
       <x:c r="D19" s="11"/>
@@ -1325,8 +1274,8 @@
       <x:c r="A20" s="3">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B20" s="1" t="s">
-        <x:v>29</x:v>
+      <x:c r="B20" s="1" t="str">
+        <x:v>Wurkz Ice ORD</x:v>
       </x:c>
       <x:c r="C20" s="10"/>
       <x:c r="D20" s="11"/>
@@ -1358,9 +1307,7 @@
       <x:c r="A21" s="3">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="s">
-        <x:v>30</x:v>
-      </x:c>
+      <x:c r="B21" s="1"/>
       <x:c r="C21" s="10"/>
       <x:c r="D21" s="11"/>
       <x:c r="E21" s="11"/>
@@ -1391,8 +1338,8 @@
       <x:c r="A22" s="3">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B22" s="1" t="s">
-        <x:v>31</x:v>
+      <x:c r="B22" s="1" t="str">
+        <x:v>CAMBODIA Sport 500mL ORD</x:v>
       </x:c>
       <x:c r="C22" s="10"/>
       <x:c r="D22" s="11"/>
@@ -1425,7 +1372,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C23" s="10"/>
       <x:c r="D23" s="11"/>
@@ -1458,7 +1405,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C24" s="10"/>
       <x:c r="D24" s="11"/>
@@ -1488,7 +1435,7 @@
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="13" t="s">
-        <x:v>34</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B25" s="9"/>
       <x:c r="C25" s="9"/>
@@ -1519,85 +1466,85 @@
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="4" t="s">
-        <x:v>35</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E26" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F26" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G26" s="4" t="s">
-        <x:v>40</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="I26" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K26" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L26" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="N26" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="O26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="P26" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="Q26" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="R26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="S26" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="T26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="U26" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="V26" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="W26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="X26" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="Y26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="Z26" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="AA26" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
@@ -1613,21 +1560,21 @@
       <x:c r="F27" s="3"/>
       <x:c r="G27" s="3"/>
       <x:c r="H27" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="I27" s="3"/>
       <x:c r="J27" s="3"/>
       <x:c r="K27" s="3"/>
       <x:c r="L27" s="3"/>
       <x:c r="M27" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="N27" s="3"/>
       <x:c r="O27" s="3"/>
       <x:c r="P27" s="3"/>
       <x:c r="Q27" s="3"/>
       <x:c r="R27" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="S27" s="3"/>
       <x:c r="T27" s="3"/>
@@ -1659,14 +1606,14 @@
       <x:c r="K28" s="3"/>
       <x:c r="L28" s="3"/>
       <x:c r="M28" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="N28" s="3"/>
       <x:c r="O28" s="3"/>
       <x:c r="P28" s="3"/>
       <x:c r="Q28" s="3"/>
       <x:c r="R28" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S28" s="3"/>
       <x:c r="T28" s="3"/>
@@ -1691,28 +1638,28 @@
       <x:c r="F29" s="3"/>
       <x:c r="G29" s="3"/>
       <x:c r="H29" s="1" t="s">
-        <x:v>46</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I29" s="3"/>
       <x:c r="J29" s="3"/>
       <x:c r="K29" s="3"/>
       <x:c r="L29" s="3"/>
       <x:c r="M29" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="N29" s="3"/>
       <x:c r="O29" s="3"/>
       <x:c r="P29" s="3"/>
       <x:c r="Q29" s="3"/>
       <x:c r="R29" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="S29" s="3"/>
       <x:c r="T29" s="3"/>
       <x:c r="U29" s="3"/>
       <x:c r="V29" s="3"/>
       <x:c r="W29" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="X29" s="3"/>
       <x:c r="Y29" s="3"/>
@@ -1737,7 +1684,7 @@
       <x:c r="K30" s="3"/>
       <x:c r="L30" s="3"/>
       <x:c r="M30" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N30" s="3"/>
       <x:c r="O30" s="3"/>
@@ -1759,7 +1706,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C31" s="3"/>
       <x:c r="D31" s="3"/>
@@ -1767,7 +1714,7 @@
       <x:c r="F31" s="3"/>
       <x:c r="G31" s="3"/>
       <x:c r="H31" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="I31" s="3"/>
       <x:c r="J31" s="3"/>
@@ -1801,8 +1748,8 @@
       <x:c r="E32" s="3"/>
       <x:c r="F32" s="3"/>
       <x:c r="G32" s="3"/>
-      <x:c r="H32" s="1" t="s">
-        <x:v>53</x:v>
+      <x:c r="H32" s="1" t="str">
+        <x:v>Boostrong ORD</x:v>
       </x:c>
       <x:c r="I32" s="3"/>
       <x:c r="J32" s="3"/>
@@ -1813,8 +1760,8 @@
       <x:c r="O32" s="3"/>
       <x:c r="P32" s="3"/>
       <x:c r="Q32" s="3"/>
-      <x:c r="R32" s="1" t="s">
-        <x:v>54</x:v>
+      <x:c r="R32" s="1" t="str">
+        <x:v>Krud ED ORD</x:v>
       </x:c>
       <x:c r="S32" s="3"/>
       <x:c r="T32" s="3"/>
@@ -1830,30 +1777,30 @@
       <x:c r="A33" s="3">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B33" s="1" t="s">
-        <x:v>29</x:v>
+      <x:c r="B33" s="1" t="str">
+        <x:v>Wurkz Ice ORD</x:v>
       </x:c>
       <x:c r="C33" s="3"/>
       <x:c r="D33" s="3"/>
       <x:c r="E33" s="3"/>
       <x:c r="F33" s="3"/>
       <x:c r="G33" s="3"/>
-      <x:c r="H33" s="1" t="s">
-        <x:v>55</x:v>
+      <x:c r="H33" s="1" t="str">
+        <x:v>Champion ORD</x:v>
       </x:c>
       <x:c r="I33" s="3"/>
       <x:c r="J33" s="3"/>
       <x:c r="K33" s="3"/>
       <x:c r="L33" s="3"/>
-      <x:c r="M33" s="1" t="s">
-        <x:v>56</x:v>
+      <x:c r="M33" s="1" t="str">
+        <x:v>King Kong Ice ORD</x:v>
       </x:c>
       <x:c r="N33" s="3"/>
       <x:c r="O33" s="3"/>
       <x:c r="P33" s="3"/>
       <x:c r="Q33" s="3"/>
-      <x:c r="R33" s="1" t="s">
-        <x:v>57</x:v>
+      <x:c r="R33" s="1" t="str">
+        <x:v>Krud Ice ORD</x:v>
       </x:c>
       <x:c r="S33" s="3"/>
       <x:c r="T33" s="3"/>
@@ -1869,30 +1816,30 @@
       <x:c r="A34" s="3">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B34" s="1" t="s">
-        <x:v>23</x:v>
+      <x:c r="B34" s="1" t="str">
+        <x:v>CAMBODIA ED ORD</x:v>
       </x:c>
       <x:c r="C34" s="3"/>
       <x:c r="D34" s="3"/>
       <x:c r="E34" s="3"/>
       <x:c r="F34" s="3"/>
       <x:c r="G34" s="3"/>
-      <x:c r="H34" s="1" t="s">
-        <x:v>58</x:v>
+      <x:c r="H34" s="1" t="str">
+        <x:v>Super Boostrong ORD</x:v>
       </x:c>
       <x:c r="I34" s="3"/>
       <x:c r="J34" s="3"/>
       <x:c r="K34" s="3"/>
       <x:c r="L34" s="3"/>
-      <x:c r="M34" s="1" t="s">
-        <x:v>59</x:v>
+      <x:c r="M34" s="1" t="str">
+        <x:v>King Kong ORD</x:v>
       </x:c>
       <x:c r="N34" s="3"/>
       <x:c r="O34" s="3"/>
       <x:c r="P34" s="3"/>
       <x:c r="Q34" s="3"/>
       <x:c r="R34" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="S34" s="3"/>
       <x:c r="T34" s="3"/>
@@ -1908,8 +1855,8 @@
       <x:c r="A35" s="3">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B35" s="1" t="s">
-        <x:v>24</x:v>
+      <x:c r="B35" s="1" t="str">
+        <x:v>DAZZ ORD</x:v>
       </x:c>
       <x:c r="C35" s="3"/>
       <x:c r="D35" s="3"/>
@@ -1917,7 +1864,7 @@
       <x:c r="F35" s="3"/>
       <x:c r="G35" s="3"/>
       <x:c r="H35" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="I35" s="3"/>
       <x:c r="J35" s="3"/>
@@ -1929,7 +1876,7 @@
       <x:c r="P35" s="3"/>
       <x:c r="Q35" s="3"/>
       <x:c r="R35" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="S35" s="3"/>
       <x:c r="T35" s="3"/>
@@ -1945,8 +1892,8 @@
       <x:c r="A36" s="3">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B36" s="1" t="s">
-        <x:v>25</x:v>
+      <x:c r="B36" s="1" t="str">
+        <x:v>DAZZ Zero Sugar ORD</x:v>
       </x:c>
       <x:c r="C36" s="3"/>
       <x:c r="D36" s="3"/>
@@ -1954,7 +1901,7 @@
       <x:c r="F36" s="3"/>
       <x:c r="G36" s="3"/>
       <x:c r="H36" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I36" s="3"/>
       <x:c r="J36" s="3"/>
@@ -1981,7 +1928,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C37" s="3"/>
       <x:c r="D37" s="3"/>
@@ -1989,7 +1936,7 @@
       <x:c r="F37" s="3"/>
       <x:c r="G37" s="3"/>
       <x:c r="H37" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="I37" s="3"/>
       <x:c r="J37" s="3"/>
@@ -2001,7 +1948,7 @@
       <x:c r="P37" s="3"/>
       <x:c r="Q37" s="3"/>
       <x:c r="R37" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="S37" s="3"/>
       <x:c r="T37" s="3"/>
@@ -2018,7 +1965,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C38" s="3"/>
       <x:c r="D38" s="3"/>
@@ -2026,14 +1973,14 @@
       <x:c r="F38" s="3"/>
       <x:c r="G38" s="3"/>
       <x:c r="H38" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="I38" s="3"/>
       <x:c r="J38" s="3"/>
       <x:c r="K38" s="3"/>
       <x:c r="L38" s="3"/>
       <x:c r="M38" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="N38" s="3"/>
       <x:c r="O38" s="3"/>
@@ -2054,30 +2001,30 @@
       <x:c r="A39" s="3">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B39" s="1" t="s">
-        <x:v>28</x:v>
+      <x:c r="B39" s="1" t="str">
+        <x:v>EXPREZ Melon ORD</x:v>
       </x:c>
       <x:c r="C39" s="3"/>
       <x:c r="D39" s="3"/>
       <x:c r="E39" s="3"/>
       <x:c r="F39" s="3"/>
       <x:c r="G39" s="3"/>
-      <x:c r="H39" s="1" t="s">
-        <x:v>69</x:v>
+      <x:c r="H39" s="1" t="str">
+        <x:v>EXPREZ Can 330ml ORD</x:v>
       </x:c>
       <x:c r="I39" s="3"/>
       <x:c r="J39" s="3"/>
       <x:c r="K39" s="3"/>
       <x:c r="L39" s="3"/>
       <x:c r="M39" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="N39" s="3"/>
       <x:c r="O39" s="3"/>
       <x:c r="P39" s="3"/>
       <x:c r="Q39" s="3"/>
-      <x:c r="R39" s="1" t="s">
-        <x:v>71</x:v>
+      <x:c r="R39" s="1" t="str">
+        <x:v>Idol Can 330ml ORD</x:v>
       </x:c>
       <x:c r="S39" s="3"/>
       <x:c r="T39" s="3"/>
@@ -2094,29 +2041,27 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C40" s="3"/>
       <x:c r="D40" s="3"/>
       <x:c r="E40" s="3"/>
       <x:c r="F40" s="3"/>
       <x:c r="G40" s="3"/>
-      <x:c r="H40" s="1" t="s">
-        <x:v>73</x:v>
-      </x:c>
+      <x:c r="H40" s="1"/>
       <x:c r="I40" s="3"/>
       <x:c r="J40" s="3"/>
       <x:c r="K40" s="3"/>
       <x:c r="L40" s="3"/>
       <x:c r="M40" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="N40" s="3"/>
       <x:c r="O40" s="3"/>
       <x:c r="P40" s="3"/>
       <x:c r="Q40" s="3"/>
       <x:c r="R40" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="S40" s="3"/>
       <x:c r="T40" s="3"/>
@@ -2133,7 +2078,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C41" s="3"/>
       <x:c r="D41" s="3"/>
@@ -2141,28 +2086,28 @@
       <x:c r="F41" s="3"/>
       <x:c r="G41" s="3"/>
       <x:c r="H41" s="1" t="s">
-        <x:v>76</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="I41" s="3"/>
       <x:c r="J41" s="3"/>
       <x:c r="K41" s="3"/>
       <x:c r="L41" s="3"/>
       <x:c r="M41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="N41" s="3"/>
       <x:c r="O41" s="3"/>
       <x:c r="P41" s="3"/>
       <x:c r="Q41" s="3"/>
       <x:c r="R41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="S41" s="3"/>
       <x:c r="T41" s="3"/>
       <x:c r="U41" s="3"/>
       <x:c r="V41" s="3"/>
       <x:c r="W41" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="X41" s="3"/>
       <x:c r="Y41" s="3"/>
@@ -2174,7 +2119,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C42" s="3"/>
       <x:c r="D42" s="3"/>
@@ -2182,28 +2127,28 @@
       <x:c r="F42" s="3"/>
       <x:c r="G42" s="3"/>
       <x:c r="H42" s="1" t="s">
-        <x:v>80</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="I42" s="3"/>
       <x:c r="J42" s="3"/>
       <x:c r="K42" s="3"/>
       <x:c r="L42" s="3"/>
       <x:c r="M42" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="N42" s="3"/>
       <x:c r="O42" s="3"/>
       <x:c r="P42" s="3"/>
       <x:c r="Q42" s="3"/>
       <x:c r="R42" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="S42" s="3"/>
       <x:c r="T42" s="3"/>
       <x:c r="U42" s="3"/>
       <x:c r="V42" s="3"/>
       <x:c r="W42" s="1" t="s">
-        <x:v>83</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="X42" s="3"/>
       <x:c r="Y42" s="3"/>
@@ -2227,7 +2172,7 @@
       <x:c r="F44" s="21"/>
       <x:c r="G44" s="12"/>
       <x:c r="I44" s="19" t="s">
-        <x:v>84</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="J44" s="9"/>
       <x:c r="K44" s="9"/>
@@ -2238,7 +2183,7 @@
       <x:c r="P44" s="9"/>
       <x:c r="Q44" s="9"/>
       <x:c r="S44" s="19" t="s">
-        <x:v>85</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="T44" s="9"/>
       <x:c r="U44" s="9"/>
@@ -2289,7 +2234,7 @@
       <x:c r="F46" s="10"/>
       <x:c r="G46" s="12"/>
       <x:c r="I46" s="13" t="s">
-        <x:v>86</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="J46" s="9"/>
       <x:c r="K46" s="9"/>
@@ -2320,7 +2265,7 @@
       <x:c r="F47" s="8"/>
       <x:c r="G47" s="9"/>
       <x:c r="I47" s="13" t="s">
-        <x:v>87</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J47" s="9"/>
       <x:c r="K47" s="9"/>
@@ -2351,7 +2296,7 @@
       <x:c r="F48" s="8"/>
       <x:c r="G48" s="9"/>
       <x:c r="I48" s="13" t="s">
-        <x:v>88</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J48" s="9"/>
       <x:c r="K48" s="9"/>
@@ -2362,7 +2307,7 @@
       <x:c r="P48" s="9"/>
       <x:c r="Q48" s="9"/>
       <x:c r="S48" s="13" t="s">
-        <x:v>88</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="T48" s="9"/>
       <x:c r="U48" s="9"/>
@@ -2534,6 +2479,6 @@
     <x:mergeCell ref="A48:G48"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e0133d9d1794866"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c2f77274d224145"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update WURKZ and Dragon ORD and restore weekly guidance
</commit_message>
<xml_diff>
--- a/templates/template_by_dealer.xlsx
+++ b/templates/template_by_dealer.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simaple_form" sheetId="1" r:id="R22278b7ba29a46f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simaple_form" sheetId="1" r:id="R3ff5319731544805"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -76,9 +76,6 @@
     <x:t xml:space="preserve">CAMBODIA COLA</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">WURKZ</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">IZE PET 300ml Flavour</x:t>
   </x:si>
   <x:si>
@@ -152,9 +149,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">BACCHUSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Dragon</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">BACCHUSE Sugar Free</x:t>
@@ -412,7 +406,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra885a6d504c24f93"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R38eff954dcf240df"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1043,8 +1037,8 @@
       <x:c r="A13" s="3">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="s">
-        <x:v>22</x:v>
+      <x:c r="B13" s="1" t="str">
+        <x:v>WURKZ ORD</x:v>
       </x:c>
       <x:c r="C13" s="10"/>
       <x:c r="D13" s="11"/>
@@ -1176,7 +1170,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C17" s="10"/>
       <x:c r="D17" s="11"/>
@@ -1209,7 +1203,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C18" s="10"/>
       <x:c r="D18" s="11"/>
@@ -1372,7 +1366,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C23" s="10"/>
       <x:c r="D23" s="11"/>
@@ -1405,7 +1399,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C24" s="10"/>
       <x:c r="D24" s="11"/>
@@ -1435,7 +1429,7 @@
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="13" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B25" s="9"/>
       <x:c r="C25" s="9"/>
@@ -1466,85 +1460,85 @@
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="s">
+      <x:c r="E26" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E26" s="4" t="s">
+      <x:c r="F26" s="4" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="F26" s="4" t="s">
+      <x:c r="G26" s="4" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="G26" s="4" t="s">
-        <x:v>33</x:v>
       </x:c>
       <x:c r="H26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="I26" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="J26" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="J26" s="4" t="s">
+      <x:c r="K26" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K26" s="4" t="s">
+      <x:c r="L26" s="4" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="L26" s="4" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="M26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="N26" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="O26" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="O26" s="4" t="s">
+      <x:c r="P26" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="P26" s="4" t="s">
+      <x:c r="Q26" s="4" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="Q26" s="4" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="R26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="S26" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="T26" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="T26" s="4" t="s">
+      <x:c r="U26" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="U26" s="4" t="s">
+      <x:c r="V26" s="4" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="V26" s="4" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="W26" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="X26" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="Y26" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="Y26" s="4" t="s">
+      <x:c r="Z26" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="Z26" s="4" t="s">
+      <x:c r="AA26" s="4" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="AA26" s="4" t="s">
-        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
@@ -1560,21 +1554,21 @@
       <x:c r="F27" s="3"/>
       <x:c r="G27" s="3"/>
       <x:c r="H27" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="I27" s="3"/>
       <x:c r="J27" s="3"/>
       <x:c r="K27" s="3"/>
       <x:c r="L27" s="3"/>
       <x:c r="M27" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="N27" s="3"/>
       <x:c r="O27" s="3"/>
       <x:c r="P27" s="3"/>
       <x:c r="Q27" s="3"/>
       <x:c r="R27" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="S27" s="3"/>
       <x:c r="T27" s="3"/>
@@ -1606,14 +1600,14 @@
       <x:c r="K28" s="3"/>
       <x:c r="L28" s="3"/>
       <x:c r="M28" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="N28" s="3"/>
       <x:c r="O28" s="3"/>
       <x:c r="P28" s="3"/>
       <x:c r="Q28" s="3"/>
       <x:c r="R28" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="S28" s="3"/>
       <x:c r="T28" s="3"/>
@@ -1638,28 +1632,28 @@
       <x:c r="F29" s="3"/>
       <x:c r="G29" s="3"/>
       <x:c r="H29" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="I29" s="3"/>
       <x:c r="J29" s="3"/>
       <x:c r="K29" s="3"/>
       <x:c r="L29" s="3"/>
       <x:c r="M29" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="N29" s="3"/>
       <x:c r="O29" s="3"/>
       <x:c r="P29" s="3"/>
       <x:c r="Q29" s="3"/>
       <x:c r="R29" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="S29" s="3"/>
       <x:c r="T29" s="3"/>
       <x:c r="U29" s="3"/>
       <x:c r="V29" s="3"/>
       <x:c r="W29" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="X29" s="3"/>
       <x:c r="Y29" s="3"/>
@@ -1684,7 +1678,7 @@
       <x:c r="K30" s="3"/>
       <x:c r="L30" s="3"/>
       <x:c r="M30" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="N30" s="3"/>
       <x:c r="O30" s="3"/>
@@ -1706,7 +1700,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C31" s="3"/>
       <x:c r="D31" s="3"/>
@@ -1714,7 +1708,7 @@
       <x:c r="F31" s="3"/>
       <x:c r="G31" s="3"/>
       <x:c r="H31" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="I31" s="3"/>
       <x:c r="J31" s="3"/>
@@ -1740,8 +1734,8 @@
       <x:c r="A32" s="3">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B32" s="1" t="s">
-        <x:v>22</x:v>
+      <x:c r="B32" s="1" t="str">
+        <x:v>WURKZ ORD</x:v>
       </x:c>
       <x:c r="C32" s="3"/>
       <x:c r="D32" s="3"/>
@@ -1839,7 +1833,7 @@
       <x:c r="P34" s="3"/>
       <x:c r="Q34" s="3"/>
       <x:c r="R34" s="1" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="S34" s="3"/>
       <x:c r="T34" s="3"/>
@@ -1864,7 +1858,7 @@
       <x:c r="F35" s="3"/>
       <x:c r="G35" s="3"/>
       <x:c r="H35" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="I35" s="3"/>
       <x:c r="J35" s="3"/>
@@ -1875,8 +1869,8 @@
       <x:c r="O35" s="3"/>
       <x:c r="P35" s="3"/>
       <x:c r="Q35" s="3"/>
-      <x:c r="R35" s="1" t="s">
-        <x:v>48</x:v>
+      <x:c r="R35" s="1" t="str">
+        <x:v>Dragon ORD</x:v>
       </x:c>
       <x:c r="S35" s="3"/>
       <x:c r="T35" s="3"/>
@@ -1901,7 +1895,7 @@
       <x:c r="F36" s="3"/>
       <x:c r="G36" s="3"/>
       <x:c r="H36" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="I36" s="3"/>
       <x:c r="J36" s="3"/>
@@ -1928,7 +1922,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C37" s="3"/>
       <x:c r="D37" s="3"/>
@@ -1936,7 +1930,7 @@
       <x:c r="F37" s="3"/>
       <x:c r="G37" s="3"/>
       <x:c r="H37" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I37" s="3"/>
       <x:c r="J37" s="3"/>
@@ -1948,7 +1942,7 @@
       <x:c r="P37" s="3"/>
       <x:c r="Q37" s="3"/>
       <x:c r="R37" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="S37" s="3"/>
       <x:c r="T37" s="3"/>
@@ -1965,7 +1959,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C38" s="3"/>
       <x:c r="D38" s="3"/>
@@ -1973,14 +1967,14 @@
       <x:c r="F38" s="3"/>
       <x:c r="G38" s="3"/>
       <x:c r="H38" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="I38" s="3"/>
       <x:c r="J38" s="3"/>
       <x:c r="K38" s="3"/>
       <x:c r="L38" s="3"/>
       <x:c r="M38" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="N38" s="3"/>
       <x:c r="O38" s="3"/>
@@ -2017,7 +2011,7 @@
       <x:c r="K39" s="3"/>
       <x:c r="L39" s="3"/>
       <x:c r="M39" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="N39" s="3"/>
       <x:c r="O39" s="3"/>
@@ -2041,7 +2035,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>56</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C40" s="3"/>
       <x:c r="D40" s="3"/>
@@ -2054,14 +2048,14 @@
       <x:c r="K40" s="3"/>
       <x:c r="L40" s="3"/>
       <x:c r="M40" s="1" t="s">
-        <x:v>57</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="N40" s="3"/>
       <x:c r="O40" s="3"/>
       <x:c r="P40" s="3"/>
       <x:c r="Q40" s="3"/>
       <x:c r="R40" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="S40" s="3"/>
       <x:c r="T40" s="3"/>
@@ -2078,7 +2072,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C41" s="3"/>
       <x:c r="D41" s="3"/>
@@ -2086,28 +2080,28 @@
       <x:c r="F41" s="3"/>
       <x:c r="G41" s="3"/>
       <x:c r="H41" s="1" t="s">
-        <x:v>59</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="I41" s="3"/>
       <x:c r="J41" s="3"/>
       <x:c r="K41" s="3"/>
       <x:c r="L41" s="3"/>
       <x:c r="M41" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="N41" s="3"/>
       <x:c r="O41" s="3"/>
       <x:c r="P41" s="3"/>
       <x:c r="Q41" s="3"/>
       <x:c r="R41" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="S41" s="3"/>
       <x:c r="T41" s="3"/>
       <x:c r="U41" s="3"/>
       <x:c r="V41" s="3"/>
       <x:c r="W41" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="X41" s="3"/>
       <x:c r="Y41" s="3"/>
@@ -2119,7 +2113,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C42" s="3"/>
       <x:c r="D42" s="3"/>
@@ -2127,28 +2121,28 @@
       <x:c r="F42" s="3"/>
       <x:c r="G42" s="3"/>
       <x:c r="H42" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="I42" s="3"/>
       <x:c r="J42" s="3"/>
       <x:c r="K42" s="3"/>
       <x:c r="L42" s="3"/>
       <x:c r="M42" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="N42" s="3"/>
       <x:c r="O42" s="3"/>
       <x:c r="P42" s="3"/>
       <x:c r="Q42" s="3"/>
       <x:c r="R42" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="S42" s="3"/>
       <x:c r="T42" s="3"/>
       <x:c r="U42" s="3"/>
       <x:c r="V42" s="3"/>
       <x:c r="W42" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="X42" s="3"/>
       <x:c r="Y42" s="3"/>
@@ -2172,7 +2166,7 @@
       <x:c r="F44" s="21"/>
       <x:c r="G44" s="12"/>
       <x:c r="I44" s="19" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J44" s="9"/>
       <x:c r="K44" s="9"/>
@@ -2183,7 +2177,7 @@
       <x:c r="P44" s="9"/>
       <x:c r="Q44" s="9"/>
       <x:c r="S44" s="19" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="T44" s="9"/>
       <x:c r="U44" s="9"/>
@@ -2234,7 +2228,7 @@
       <x:c r="F46" s="10"/>
       <x:c r="G46" s="12"/>
       <x:c r="I46" s="13" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="J46" s="9"/>
       <x:c r="K46" s="9"/>
@@ -2265,7 +2259,7 @@
       <x:c r="F47" s="8"/>
       <x:c r="G47" s="9"/>
       <x:c r="I47" s="13" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J47" s="9"/>
       <x:c r="K47" s="9"/>
@@ -2296,7 +2290,7 @@
       <x:c r="F48" s="8"/>
       <x:c r="G48" s="9"/>
       <x:c r="I48" s="13" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="J48" s="9"/>
       <x:c r="K48" s="9"/>
@@ -2307,7 +2301,7 @@
       <x:c r="P48" s="9"/>
       <x:c r="Q48" s="9"/>
       <x:c r="S48" s="13" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="T48" s="9"/>
       <x:c r="U48" s="9"/>
@@ -2479,6 +2473,6 @@
     <x:mergeCell ref="A48:G48"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c2f77274d224145"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re850858ad086476b"/>
 </x:worksheet>
 </file>
</xml_diff>